<commit_message>
pupil analysis and drug inhibition
</commit_message>
<xml_diff>
--- a/matlabCode/operantMatching/learningModels/stan/stanParams.xlsx
+++ b/matlabCode/operantMatching/learningModels/stan/stanParams.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22624"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cooper_PC\Desktop\githubRepositories\cooperAnalysis\matlabCode\operantMatching\learningModels\stan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zhixi\Documents\gitRepositories\sueAnalysis\matlabCode\operantMatching\learningModels\stan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BFB5040-6037-4752-A068-CCA069E98A9B}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8413DE6B-D633-4E68-AE37-4D70378BAEFB}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" activeTab="1" xr2:uid="{4D34CB12-A0A6-45A3-A487-E26274108661}"/>
+    <workbookView xWindow="-15390" yWindow="3345" windowWidth="15120" windowHeight="9435" activeTab="4" xr2:uid="{4D34CB12-A0A6-45A3-A487-E26274108661}"/>
   </bookViews>
   <sheets>
     <sheet name="CG09" sheetId="3" r:id="rId1"/>
     <sheet name="CG14" sheetId="1" r:id="rId2"/>
     <sheet name="CG15" sheetId="2" r:id="rId3"/>
     <sheet name="CG16" sheetId="4" r:id="rId4"/>
+    <sheet name="combine" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
   <si>
     <t>fiveParamOFixed</t>
   </si>
@@ -46,6 +47,12 @@
   </si>
   <si>
     <t>fiveParamOfourStart_preS_aFboth</t>
+  </si>
+  <si>
+    <t>fourParamForDrug</t>
+  </si>
+  <si>
+    <t>fourParamForSaline</t>
   </si>
 </sst>
 </file>
@@ -623,4 +630,57 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6360FF7-4C61-451D-98B3-2CB066FE049E}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0.40751500000000002</v>
+      </c>
+      <c r="B2">
+        <v>0.40751500000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>0.52324499999999996</v>
+      </c>
+      <c r="B3">
+        <v>0.52324499999999996</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>0.382546</v>
+      </c>
+      <c r="B4">
+        <v>0.382546</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4.1933400000000001</v>
+      </c>
+      <c r="B5">
+        <v>4.1933400000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>